<commit_message>
Release v0.3.0 - Project Management & UX Improvements
Major improvements:
- Move backup and deleted files to hidden subdirectories (.backups, .trash)
- Auto-reload radar when switching from edit to view mode
- Auto-increment duplicate entry names (New Entry 2, 3, etc.)

Changes:
- Backup files now stored in .backups/ subdirectory instead of cluttering project folder
- Deleted files now stored in .trash/ subdirectory
- Radar visualization automatically refreshes when switching to view mode
- Adding new entries now generates unique names to prevent duplicates
- Updated backup_manager.py and api.py to use new directory structure

Fixes:
- Fixed radar not updating after editing in Excel mode
- Fixed duplicate name validation errors when adding multiple entries
- Cleaned up project folder by hiding system files
</commit_message>
<xml_diff>
--- a/templates/radar_template.xlsx
+++ b/templates/radar_template.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -26,30 +27,20 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
+      <color rgb="00FFFFFF"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color rgb="FF4472C4"/>
+      <color rgb="004472C4"/>
       <sz val="16"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -61,14 +52,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4472C4"/>
-        <bgColor rgb="FF4472C4"/>
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE7E6E6"/>
-        <bgColor rgb="FFE7E6E6"/>
+        <fgColor rgb="00E7E6E6"/>
+        <bgColor rgb="00E7E6E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -84,18 +75,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -458,14 +448,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" style="5" min="1" max="1"/>
-    <col width="20" customWidth="1" style="5" min="2" max="4"/>
-    <col width="60" customWidth="1" style="5" min="5" max="5"/>
-    <col width="20" customWidth="1" style="5" min="6" max="6"/>
-    <col width="25" customWidth="1" style="5" min="7" max="8"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -486,42 +480,32 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>dealSize</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>propensityToWin</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>isStrategic</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>tags</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>link</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>linkName</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>dealSize</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>propensityToWin</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>isStrategic</t>
         </is>
       </c>
     </row>
@@ -533,7 +517,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Current HY</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -543,25 +527,30 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>On Track</t>
+          <t>&gt; $500k</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>&lt;p&gt;Comprehensive strategy for migrating legacy applications to cloud infrastructure. Includes assessment, planning, and execution phases.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>cloud, migration, infrastructure</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>https://example.com/cloud-strategy</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>View Strategy Doc</t>
         </is>
@@ -575,35 +564,40 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Next HY</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Applications</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>$100k - $500k</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>&lt;p&gt;Next-generation analytics platform leveraging &lt;strong&gt;machine learning&lt;/strong&gt; and AI to provide predictive insights.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>AI, analytics, machine-learning</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>https://example.com/ai-analytics</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Platform Overview</t>
         </is>
@@ -612,51 +606,58 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Quantum Computing Research</t>
+          <t>Process Automation Initiative</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Year +1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Emerging Tech</t>
+          <t>Automation</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>&lt; $100k</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Long-term research initiative exploring quantum computing applications for optimization problems.&lt;/p&gt;</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>quantum, research, innovation</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Initiative to automate manual business processes using RPA and workflow automation tools.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Status" error="Please select a valid status value" type="list">
-      <formula1>"On Track,At Risk,Blocked,New,Moved In,Moved Out"</formula1>
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid Ring" error="Please select a valid ring value" type="list">
+      <formula1>"Current HY,Next HY,Year +1,Year +2"</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid Ring" error="Please select a valid ring value" type="list">
-      <formula1>"Q1,Q2,Q3,Q4,Beyond"</formula1>
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid Quadrant" error="Please select a valid quadrant value" type="list">
+      <formula1>"Automation,Data,Infrastructure"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Deal Size" error="Please select a valid deal size" promptTitle="Deal Size" prompt="Select deal size category" type="list">
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Deal Size" error="Please select a valid deal size" type="list">
       <formula1>"&lt; $100k,$100k - $500k,&gt; $500k"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Propensity" error="Please select from the list" type="list">
+    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Propensity" error="Please select a valid propensity to win" type="list">
       <formula1>"Low,Medium,High"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Value" error="Please select TRUE or FALSE" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
+    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Strategic Value" error="Please select Yes or No" type="list">
+      <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -669,24 +670,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <dimension ref="A1:D38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" style="5" min="1" max="1"/>
-    <col width="12" customWidth="1" style="5" min="2" max="2"/>
-    <col width="60" customWidth="1" style="5" min="3" max="3"/>
-    <col width="30" customWidth="1" style="5" min="4" max="4"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" customHeight="1" s="5">
-      <c r="A1" s="4" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Radar Studio - Import Template Instructions</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="19" customHeight="1" s="5">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Overview</t>
         </is>
@@ -706,30 +707,30 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="19" customHeight="1" s="5">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Column Descriptions</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Example</t>
         </is>
@@ -770,12 +771,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Time horizon: Q1, Q2, Q3, Q4, Beyond This Year</t>
+          <t>Time horizon: Current HY, Next HY, Year +1, Year +2</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Current HY</t>
         </is>
       </c>
     </row>
@@ -792,7 +793,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Category/domain (flexible, can be any text)</t>
+          <t>Category: Automation, Data, or Infrastructure</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -804,7 +805,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>dealSize</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -814,19 +815,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Current status: On Track, At Risk, Blocked, New, Moved In, Moved Out</t>
+          <t>Deal size category: &lt; $100k, $100k - $500k, &gt; $500k</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>On Track</t>
+          <t>&gt; $500k</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>propensityToWin</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -836,19 +837,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>HTML description (supports &lt;p&gt;, &lt;strong&gt;, &lt;em&gt;, &lt;a&gt;, &lt;ul&gt;, &lt;li&gt;)</t>
+          <t>Likelihood to win: Low, Medium, High</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Detailed description...&lt;/p&gt;</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>tags</t>
+          <t>isStrategic</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -858,19 +859,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Comma-separated tags for filtering</t>
+          <t>Strategic importance: Yes or No (shows star indicator)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>cloud, migration, infrastructure</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>link</t>
+          <t>description</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -880,19 +881,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>URL for external reference</t>
+          <t>HTML description (supports &lt;p&gt;, &lt;strong&gt;, &lt;em&gt;, &lt;a&gt;, &lt;ul&gt;, &lt;li&gt;)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://example.com/doc</t>
+          <t>&lt;p&gt;Detailed description...&lt;/p&gt;</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>linkName</t>
+          <t>link</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -902,19 +903,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Display text for the link</t>
+          <t>URL for external reference</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>View Documentation</t>
+          <t>https://example.com/doc</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>dealSize</t>
+          <t>linkName</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -924,18 +925,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Deal size category: &lt; $100k, $100k - $500k, &gt; $500k</t>
+          <t>Display text for the link</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>$100k - $500k</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="19" customHeight="1" s="5"/>
+          <t>View Documentation</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>How to Import</t>
         </is>
@@ -951,14 +951,14 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2. Use the dropdown menus for Ring and Status columns</t>
+          <t>2. Use the dropdown menus for Ring, Quadrant, Deal Size, Propensity, and Strategic columns</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3. Type any value you want for Quadrant (free text)</t>
+          <t>3. Name and Ring are required; Quadrant must be one of: Automation, Data, Infrastructure</t>
         </is>
       </c>
     </row>
@@ -990,9 +990,8 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="19" customHeight="1" s="5"/>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Tips</t>
         </is>
@@ -1008,35 +1007,42 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>• Tags help with searching and filtering - use consistent tag names</t>
+          <t>• Deal Size affects the circle size on the radar (larger deals = bigger circles)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>• Quadrants are required and flexible - create your own categories as needed</t>
+          <t>• Propensity to Win affects the circle color (High=green, Medium=yellow, Low=red)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>• Leave optional fields empty if not needed</t>
+          <t>• Strategic items show a white star in the center of the circle</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>• Ensure 'name' and 'quadrant' values are not empty</t>
+          <t>• Quadrants must be: Automation, Data, or Infrastructure</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>• Ring values must match: Ready, Less Than 1 Year, 1-3 Years, or 3+ Years</t>
+          <t>• Ring values must match: Current HY, Next HY, Year +1, or Year +2</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>• Leave optional fields empty if not needed</t>
         </is>
       </c>
     </row>

</xml_diff>